<commit_message>
Update Commands.xlsx + main.cpp
- fixed a typo, added more info to commands
- removed the address disabling for ldz from the bus transfer register, since it will disable the address bus one cycle later. This seemed too complicated, and it doesnt really matter
</commit_message>
<xml_diff>
--- a/school/Thesis Documentation/Assembler/Commands.xlsx
+++ b/school/Thesis Documentation/Assembler/Commands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Files\GitHub\Computer_HTL\school\Thesis Documentation\Assembler\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E11257DA-BA40-4E97-88D4-C5DC6075D8E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540A747C-FD31-4827-B9BD-E4F59B7969FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-3255" windowWidth="16440" windowHeight="28320" xr2:uid="{6EFB07F8-8C02-48DB-B2F6-8930B2DB515A}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="111">
   <si>
     <t>Command</t>
   </si>
@@ -308,9 +308,6 @@
     <t>Load Outputs</t>
   </si>
   <si>
-    <t>Ouput to</t>
-  </si>
-  <si>
     <t>-</t>
   </si>
   <si>
@@ -348,13 +345,37 @@
   </si>
   <si>
     <t>Outputs</t>
+  </si>
+  <si>
+    <t>Output to</t>
+  </si>
+  <si>
+    <t>Arguments</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>Address, Data</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>Reg A/B</t>
+  </si>
+  <si>
+    <t>Reg C</t>
+  </si>
+  <si>
+    <t>Reg A</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -375,6 +396,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -384,7 +413,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="19">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -604,49 +633,25 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thick">
+      <left style="medium">
         <color rgb="FF000000"/>
       </left>
       <right style="medium">
         <color rgb="FF000000"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color rgb="FF000000"/>
       </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thick">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
@@ -675,15 +680,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
@@ -693,20 +689,30 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1" readingOrder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1042,774 +1048,952 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B0EE8031-7DED-42A6-B545-7034B63A7F85}">
-  <dimension ref="F7:H86"/>
+  <dimension ref="F7:I86"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="16.28515625" customWidth="1"/>
-    <col min="7" max="7" width="29.42578125" customWidth="1"/>
-    <col min="8" max="8" width="29.85546875" customWidth="1"/>
+    <col min="7" max="7" width="20.85546875" customWidth="1"/>
+    <col min="8" max="8" width="17.28515625" customWidth="1"/>
+    <col min="9" max="9" width="25.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="6:8" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
-    <row r="8" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F8" s="10" t="s">
-        <v>92</v>
-      </c>
-      <c r="G8" s="11"/>
-      <c r="H8" s="12"/>
-    </row>
-    <row r="9" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F9" s="13" t="s">
+    <row r="7" spans="6:9" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="8" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F8" s="13" t="s">
+        <v>91</v>
+      </c>
+      <c r="G8" s="14"/>
+      <c r="H8" s="14"/>
+      <c r="I8" s="15"/>
+    </row>
+    <row r="9" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F9" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G9" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H9" s="15" t="s">
+      <c r="G9" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H9" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I9" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="6:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="6:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F10" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="G10" s="2" t="s">
-        <v>91</v>
-      </c>
-      <c r="H10" s="4" t="s">
+      <c r="G10" s="19" t="s">
+        <v>90</v>
+      </c>
+      <c r="H10" s="2" t="s">
+        <v>90</v>
+      </c>
+      <c r="I10" s="4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="11" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F11" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="G11" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H11" s="6" t="s">
+      <c r="G11" s="20" t="s">
+        <v>105</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I11" s="6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="12" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F12" s="16" t="s">
+    <row r="12" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F12" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="17" t="s">
-        <v>91</v>
-      </c>
-      <c r="H12" s="18" t="s">
+      <c r="G12" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="H12" s="8" t="s">
+        <v>90</v>
+      </c>
+      <c r="I12" s="9" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F13" s="19"/>
-      <c r="G13" s="19"/>
-      <c r="H13" s="20"/>
-    </row>
-    <row r="14" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F14" s="10" t="s">
-        <v>93</v>
-      </c>
-      <c r="G14" s="11"/>
-      <c r="H14" s="12"/>
-    </row>
-    <row r="15" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F15" s="13" t="s">
+    <row r="13" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F13" s="16"/>
+      <c r="G13" s="16"/>
+      <c r="H13" s="17"/>
+    </row>
+    <row r="14" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F14" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="G14" s="14"/>
+      <c r="H14" s="14"/>
+      <c r="I14" s="15"/>
+    </row>
+    <row r="15" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F15" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G15" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H15" s="15" t="s">
+      <c r="G15" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H15" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I15" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="6:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="6:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="F16" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="G16" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H16" s="6" t="s">
+      <c r="G16" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H16" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I16" s="6" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="17" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="17" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F17" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="G17" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H17" s="6" t="s">
+      <c r="G17" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="H17" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I17" s="6" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="18" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F18" s="5" t="s">
+    <row r="18" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F18" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="G18" s="1" t="s">
+      <c r="G18" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H18" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="H18" s="6" t="s">
+      <c r="I18" s="9" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="19" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F19" s="19"/>
-      <c r="G19" s="19"/>
-      <c r="H19" s="20"/>
-    </row>
-    <row r="20" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F20" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="G20" s="11"/>
-      <c r="H20" s="12"/>
-    </row>
-    <row r="21" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F21" s="13" t="s">
+    <row r="19" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F19" s="16"/>
+      <c r="G19" s="16"/>
+      <c r="H19" s="17"/>
+    </row>
+    <row r="20" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F20" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
+      <c r="I20" s="15"/>
+    </row>
+    <row r="21" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F21" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G21" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H21" s="15" t="s">
+      <c r="G21" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H21" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I21" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F22" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H22" s="6" t="s">
+      <c r="G22" s="19" t="s">
+        <v>106</v>
+      </c>
+      <c r="H22" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I22" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="23" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F23" s="5" t="s">
+    <row r="23" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F23" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="G23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H23" s="6" t="s">
+      <c r="G23" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="H23" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I23" s="9" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="24" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F24" s="19"/>
-      <c r="G24" s="19"/>
-      <c r="H24" s="20"/>
-    </row>
-    <row r="25" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F25" s="10" t="s">
-        <v>95</v>
-      </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="12"/>
-    </row>
-    <row r="26" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F26" s="13" t="s">
+    <row r="24" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F24" s="16"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="17"/>
+    </row>
+    <row r="25" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F25" s="13" t="s">
+        <v>94</v>
+      </c>
+      <c r="G25" s="14"/>
+      <c r="H25" s="14"/>
+      <c r="I25" s="15"/>
+    </row>
+    <row r="26" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F26" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G26" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H26" s="15" t="s">
+      <c r="G26" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H26" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I26" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F27" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="G27" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H27" s="6" t="s">
+      <c r="G27" s="19" t="s">
+        <v>108</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F28" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="G28" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H28" s="6" t="s">
+      <c r="G28" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H28" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I28" s="6" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="29" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F29" s="5" t="s">
+    <row r="29" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F29" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="G29" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H29" s="6" t="s">
+      <c r="G29" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="H29" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I29" s="9" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="30" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F30" s="19"/>
-      <c r="G30" s="19"/>
-      <c r="H30" s="20"/>
-    </row>
-    <row r="31" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F31" s="10" t="s">
-        <v>96</v>
-      </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="12"/>
-    </row>
-    <row r="32" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F32" s="13" t="s">
+    <row r="30" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F30" s="16"/>
+      <c r="G30" s="16"/>
+      <c r="H30" s="17"/>
+    </row>
+    <row r="31" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F31" s="13" t="s">
+        <v>95</v>
+      </c>
+      <c r="G31" s="14"/>
+      <c r="H31" s="14"/>
+      <c r="I31" s="15"/>
+    </row>
+    <row r="32" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F32" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G32" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H32" s="15" t="s">
+      <c r="G32" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H32" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I32" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F33" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G33" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H33" s="6" t="s">
+      <c r="G33" s="19" t="s">
+        <v>109</v>
+      </c>
+      <c r="H33" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I33" s="6" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="34" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F34" s="5" t="s">
+    <row r="34" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F34" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="G34" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H34" s="6" t="s">
+      <c r="G34" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="H34" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I34" s="9" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="35" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F35" s="19"/>
-      <c r="G35" s="19"/>
-      <c r="H35" s="20"/>
-    </row>
-    <row r="36" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F36" s="10" t="s">
-        <v>97</v>
-      </c>
-      <c r="G36" s="11"/>
-      <c r="H36" s="12"/>
-    </row>
-    <row r="37" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F37" s="13" t="s">
+    <row r="35" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F35" s="16"/>
+      <c r="G35" s="16"/>
+      <c r="H35" s="17"/>
+    </row>
+    <row r="36" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F36" s="13" t="s">
+        <v>96</v>
+      </c>
+      <c r="G36" s="14"/>
+      <c r="H36" s="14"/>
+      <c r="I36" s="15"/>
+    </row>
+    <row r="37" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F37" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G37" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H37" s="15" t="s">
+      <c r="G37" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I37" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F38" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="G38" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H38" s="6" t="s">
+      <c r="G38" s="19" t="s">
+        <v>110</v>
+      </c>
+      <c r="H38" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I38" s="6" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="39" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F39" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="G39" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H39" s="6" t="s">
+      <c r="G39" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H39" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I39" s="6" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="40" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F40" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="G40" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H40" s="6" t="s">
+      <c r="G40" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H40" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I40" s="6" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="41" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F41" s="5" t="s">
         <v>36</v>
       </c>
-      <c r="G41" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H41" s="6" t="s">
+      <c r="G41" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H41" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I41" s="6" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="42" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F42" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="G42" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H42" s="6" t="s">
+      <c r="G42" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H42" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I42" s="6" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="43" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F43" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G43" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H43" s="6" t="s">
+      <c r="G43" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H43" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I43" s="6" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="44" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F44" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="G44" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H44" s="6" t="s">
+      <c r="G44" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H44" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I44" s="6" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F45" s="5" t="s">
+    <row r="45" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F45" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="G45" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H45" s="6" t="s">
+      <c r="G45" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="H45" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I45" s="9" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="46" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F46" s="19"/>
-      <c r="G46" s="19"/>
-      <c r="H46" s="20"/>
-    </row>
-    <row r="47" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F47" s="10" t="s">
-        <v>98</v>
-      </c>
-      <c r="G47" s="11"/>
-      <c r="H47" s="12"/>
-    </row>
-    <row r="48" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F48" s="13" t="s">
+    <row r="46" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F46" s="16"/>
+      <c r="G46" s="16"/>
+      <c r="H46" s="17"/>
+    </row>
+    <row r="47" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F47" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="G47" s="14"/>
+      <c r="H47" s="14"/>
+      <c r="I47" s="15"/>
+    </row>
+    <row r="48" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F48" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G48" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H48" s="15" t="s">
+      <c r="G48" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H48" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I48" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="49" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="49" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F49" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="G49" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H49" s="6" t="s">
+      <c r="G49" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H49" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I49" s="6" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="50" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="50" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F50" s="5" t="s">
         <v>48</v>
       </c>
-      <c r="G50" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H50" s="6" t="s">
+      <c r="G50" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="H50" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I50" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F51" s="5" t="s">
+    <row r="51" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F51" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="G51" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H51" s="6" t="s">
+      <c r="G51" s="21" t="s">
+        <v>108</v>
+      </c>
+      <c r="H51" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I51" s="9" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="52" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F52" s="19"/>
-      <c r="G52" s="19"/>
-      <c r="H52" s="20"/>
-    </row>
-    <row r="53" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F53" s="10" t="s">
-        <v>99</v>
-      </c>
-      <c r="G53" s="11"/>
-      <c r="H53" s="12"/>
-    </row>
-    <row r="54" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F54" s="13" t="s">
+    <row r="52" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F52" s="16"/>
+      <c r="G52" s="16"/>
+      <c r="H52" s="17"/>
+    </row>
+    <row r="53" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F53" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="G53" s="14"/>
+      <c r="H53" s="14"/>
+      <c r="I53" s="15"/>
+    </row>
+    <row r="54" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F54" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G54" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H54" s="15" t="s">
+      <c r="G54" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H54" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I54" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="55" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="55" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F55" s="5" t="s">
         <v>52</v>
       </c>
-      <c r="G55" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H55" s="6" t="s">
+      <c r="G55" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H55" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I55" s="6" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="56" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="56" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F56" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="G56" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H56" s="6" t="s">
+      <c r="G56" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H56" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I56" s="6" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="57" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F57" s="5" t="s">
         <v>56</v>
       </c>
-      <c r="G57" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H57" s="6" t="s">
+      <c r="G57" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="H57" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I57" s="6" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="58" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="58" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F58" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="G58" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H58" s="6" t="s">
+      <c r="G58" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H58" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I58" s="6" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="59" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="59" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F59" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="G59" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H59" s="6" t="s">
+      <c r="G59" s="20" t="s">
+        <v>107</v>
+      </c>
+      <c r="H59" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I59" s="6" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="60" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F60" s="5" t="s">
+    <row r="60" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F60" s="7" t="s">
         <v>62</v>
       </c>
-      <c r="G60" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H60" s="6" t="s">
+      <c r="G60" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H60" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I60" s="9" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="61" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F61" s="19"/>
-      <c r="G61" s="19"/>
-      <c r="H61" s="20"/>
-    </row>
-    <row r="62" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F62" s="10" t="s">
-        <v>100</v>
-      </c>
-      <c r="G62" s="11"/>
-      <c r="H62" s="12"/>
-    </row>
-    <row r="63" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F63" s="13" t="s">
+    <row r="61" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F61" s="16"/>
+      <c r="G61" s="16"/>
+      <c r="H61" s="17"/>
+    </row>
+    <row r="62" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F62" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="G62" s="14"/>
+      <c r="H62" s="14"/>
+      <c r="I62" s="15"/>
+    </row>
+    <row r="63" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F63" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G63" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H63" s="15" t="s">
+      <c r="G63" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H63" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I63" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="64" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="64" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F64" s="5" t="s">
         <v>64</v>
       </c>
-      <c r="G64" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H64" s="6" t="s">
+      <c r="G64" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H64" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I64" s="6" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="65" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="65" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F65" s="5" t="s">
         <v>66</v>
       </c>
-      <c r="G65" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H65" s="6" t="s">
+      <c r="G65" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H65" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I65" s="6" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="66" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="66" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F66" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="G66" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H66" s="6" t="s">
+      <c r="G66" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H66" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I66" s="6" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="67" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F67" s="5" t="s">
+    <row r="67" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F67" s="7" t="s">
         <v>70</v>
       </c>
-      <c r="G67" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H67" s="6" t="s">
+      <c r="G67" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H67" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I67" s="9" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="68" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F68" s="19"/>
-      <c r="G68" s="19"/>
-      <c r="H68" s="20"/>
-    </row>
-    <row r="69" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F69" s="10" t="s">
-        <v>101</v>
-      </c>
-      <c r="G69" s="11"/>
-      <c r="H69" s="12"/>
-    </row>
-    <row r="70" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F70" s="13" t="s">
+    <row r="68" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F68" s="16"/>
+      <c r="G68" s="16"/>
+      <c r="H68" s="17"/>
+    </row>
+    <row r="69" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F69" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="G69" s="14"/>
+      <c r="H69" s="14"/>
+      <c r="I69" s="15"/>
+    </row>
+    <row r="70" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F70" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G70" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H70" s="15" t="s">
+      <c r="G70" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H70" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I70" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="71" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="71" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F71" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="G71" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H71" s="6" t="s">
+      <c r="G71" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H71" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I71" s="6" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="72" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="72" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F72" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="G72" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H72" s="6" t="s">
+      <c r="G72" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H72" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I72" s="6" t="s">
         <v>75</v>
       </c>
     </row>
-    <row r="73" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="73" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F73" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="G73" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H73" s="6" t="s">
+      <c r="G73" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="H73" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I73" s="6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="74" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F74" s="5" t="s">
+    <row r="74" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F74" s="7" t="s">
         <v>78</v>
       </c>
-      <c r="G74" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H74" s="6" t="s">
+      <c r="G74" s="21" t="s">
+        <v>109</v>
+      </c>
+      <c r="H74" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I74" s="9" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="75" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F75" s="19"/>
-      <c r="G75" s="19"/>
-      <c r="H75" s="20"/>
-    </row>
-    <row r="76" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F76" s="10" t="s">
-        <v>102</v>
-      </c>
-      <c r="G76" s="11"/>
-      <c r="H76" s="12"/>
-    </row>
-    <row r="77" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F77" s="13" t="s">
+    <row r="75" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F75" s="16"/>
+      <c r="G75" s="16"/>
+      <c r="H75" s="17"/>
+    </row>
+    <row r="76" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F76" s="13" t="s">
+        <v>101</v>
+      </c>
+      <c r="G76" s="14"/>
+      <c r="H76" s="14"/>
+      <c r="I76" s="15"/>
+    </row>
+    <row r="77" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F77" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="G77" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H77" s="15" t="s">
+      <c r="G77" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H77" s="11" t="s">
+        <v>103</v>
+      </c>
+      <c r="I77" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="78" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="78" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F78" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="G78" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H78" s="6" t="s">
+      <c r="G78" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H78" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I78" s="6" t="s">
         <v>81</v>
       </c>
     </row>
-    <row r="79" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="79" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F79" s="5" t="s">
         <v>82</v>
       </c>
-      <c r="G79" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H79" s="6" t="s">
+      <c r="G79" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="H79" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="I79" s="6" t="s">
         <v>83</v>
       </c>
     </row>
-    <row r="80" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F80" s="5" t="s">
+    <row r="80" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F80" s="7" t="s">
         <v>84</v>
       </c>
-      <c r="G80" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="H80" s="6" t="s">
+      <c r="G80" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H80" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I80" s="9" t="s">
         <v>85</v>
       </c>
     </row>
-    <row r="81" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F81" s="19"/>
-      <c r="G81" s="19"/>
-      <c r="H81" s="20"/>
-    </row>
-    <row r="82" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F82" s="10" t="s">
+    <row r="81" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F81" s="16"/>
+      <c r="G81" s="16"/>
+      <c r="H81" s="17"/>
+    </row>
+    <row r="82" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F82" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="G82" s="14"/>
+      <c r="H82" s="14"/>
+      <c r="I82" s="15"/>
+    </row>
+    <row r="83" spans="6:9" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F83" s="10" t="s">
+        <v>0</v>
+      </c>
+      <c r="G83" s="18" t="s">
+        <v>104</v>
+      </c>
+      <c r="H83" s="11" t="s">
         <v>103</v>
       </c>
-      <c r="G82" s="11"/>
-      <c r="H82" s="12"/>
-    </row>
-    <row r="83" spans="6:8" ht="16.5" thickTop="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="F83" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="G83" s="14" t="s">
-        <v>90</v>
-      </c>
-      <c r="H83" s="15" t="s">
+      <c r="I83" s="12" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="84" spans="6:8" x14ac:dyDescent="0.25">
+    <row r="84" spans="6:9" x14ac:dyDescent="0.25">
       <c r="F84" s="5" t="s">
         <v>86</v>
       </c>
-      <c r="G84" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="H84" s="6" t="s">
+      <c r="G84" s="19" t="s">
+        <v>107</v>
+      </c>
+      <c r="H84" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="I84" s="6" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="85" spans="6:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="6:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="F85" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="G85" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H85" s="9" t="s">
+      <c r="G85" s="21" t="s">
+        <v>90</v>
+      </c>
+      <c r="H85" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="I85" s="9" t="s">
         <v>89</v>
       </c>
     </row>
-    <row r="86" spans="6:8" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
+    <row r="86" spans="6:9" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="F31:H31"/>
-    <mergeCell ref="F8:H8"/>
-    <mergeCell ref="F14:H14"/>
-    <mergeCell ref="F20:H20"/>
-    <mergeCell ref="F25:H25"/>
-    <mergeCell ref="F82:H82"/>
-    <mergeCell ref="F36:H36"/>
-    <mergeCell ref="F47:H47"/>
-    <mergeCell ref="F53:H53"/>
-    <mergeCell ref="F62:H62"/>
-    <mergeCell ref="F69:H69"/>
-    <mergeCell ref="F76:H76"/>
+    <mergeCell ref="F36:I36"/>
+    <mergeCell ref="F47:I47"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="F62:I62"/>
+    <mergeCell ref="F69:I69"/>
+    <mergeCell ref="F76:I76"/>
+    <mergeCell ref="F82:I82"/>
+    <mergeCell ref="F8:I8"/>
+    <mergeCell ref="F14:I14"/>
+    <mergeCell ref="F20:I20"/>
+    <mergeCell ref="F25:I25"/>
+    <mergeCell ref="F31:I31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>